<commit_message>
docs: atualiza métricas da E1 e ADR-0001 com carga desduplicada (785k despesas)
Co-authored-by: bigkaio <kaio050903@gmail.com>
Co-authored-by: alvezclari <claraaalves.7@gmail.com>
Co-authored-by: Amandaaaaabreu <amandaabreu045@gmail.com>
Co-authored-by: filipe-002 <002.f1l1p3@gmail.com>
Co-authored-by: GabrielMEsteves <gabrielesteves@outlook.com>
</commit_message>
<xml_diff>
--- a/docs/projetoengenhariadedadosbd2.xlsx
+++ b/docs/projetoengenhariadedadosbd2.xlsx
@@ -1,24 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <sheets>
-    <sheet name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Identificação" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="1 Fontes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2 Formatos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="3 Modelos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="4 Cargas e Engines" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="5 Pipeline" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ADR" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Riscos" sheetId="9" state="visible" r:id="rId9"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-09-27T06:40:07Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-09-27T06:40:07Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="20">
@@ -427,7 +423,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
@@ -621,7 +617,26 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <sheets>
+    <sheet name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Identificação" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="1 Fontes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2 Formatos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="3 Modelos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="4 Cargas e Engines" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="5 Pipeline" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ADR" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Riscos" sheetId="9" state="visible" r:id="rId9"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1984,7 +1999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3157,7 +3172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4916,7 +4931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6433,7 +6448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8397,7 +8412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9828,7 +9843,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11342,7 +11357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11732,7 +11747,7 @@
       </c>
       <c r="C22" s="36" t="inlineStr">
         <is>
-          <t>Medição empírica no PostgreSQL 16: a carga dos 4 anos (921.280 linhas) levou apenas 110,7 segundos com staging COPY; o espaço ocupado foi reduzido para ~198 MB de dados limpos; a consulta agregada indexada respondeu em 115 ms contra 820 ms da tabela flat.</t>
+          <t>MediÃ§Ã£o empÃ­rica no PostgreSQL 16: a carga dos 4 anos (785.754 linhas) levou apenas 97,4 segundos com staging COPY; o espaÃ§o ocupado foi reduzido para ~178 MB de dados limpos; a consulta agregada indexada respondeu em 112 ms contra 790 ms da tabela flat.</t>
         </is>
       </c>
       <c r="D22" s="31" t="inlineStr">
@@ -12806,7 +12821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>